<commit_message>
Descarga de pdf de prueba ok
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cristian\Documents\Proyectos\F29Downloader\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\Projects\Proyectos\F29\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082E0426-D65E-44B8-A243-1388B7229BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FBABA33-DE6B-4F86-94D9-40F8754F9554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
   <si>
     <t>Rut</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>PATRICIO2018</t>
-  </si>
-  <si>
-    <t>document.querySelectorAll("#item-form")[2].childNodes[1].childNodes[0].childNodes[0].childNodes[0].childNodes[0].childNodes[0].childNodes[0].childNodes[0].childNodes[0].click()</t>
   </si>
 </sst>
 </file>
@@ -367,7 +364,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" customWidth="1"/>
@@ -375,7 +372,7 @@
     <col min="3" max="3" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -386,7 +383,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -397,7 +394,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -407,17 +404,14 @@
       <c r="C3" s="1">
         <v>46143</v>
       </c>
-      <c r="F3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C6" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
seleecion mes en excell
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\Projects\Proyectos\F29\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E20D0A-4090-477A-B02A-A288E239C6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FE29AF-82B5-4088-BC3E-7A8992560B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="3045" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
   <si>
     <t>Rut</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>Patricio2026@</t>
+  </si>
+  <si>
+    <t>05/26</t>
   </si>
 </sst>
 </file>
@@ -90,10 +93,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -401,8 +405,8 @@
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1">
-        <v>46143</v>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -412,8 +416,8 @@
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1">
-        <v>46143</v>
+      <c r="C3" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
reconocer error login y reintento
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\Projects\Proyectos\F29\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FE29AF-82B5-4088-BC3E-7A8992560B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8489BEB3-8E07-4E6E-9F1E-99C3CBD03B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="3045" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,10 +39,10 @@
     <t>76869422-2</t>
   </si>
   <si>
-    <t>Patricio2026@</t>
-  </si>
-  <si>
     <t>05/26</t>
+  </si>
+  <si>
+    <t>Patricio2026</t>
   </si>
 </sst>
 </file>
@@ -383,7 +383,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
     <col min="3" max="3" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -403,10 +403,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -414,10 +414,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -432,8 +432,8 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{CFD0AADF-4902-4B28-AE77-0F0DB06EF357}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{1B31ABDF-0568-4963-AA52-132C4AEEFDB0}"/>
+    <hyperlink ref="B2" r:id="rId1" display="Patricio2026@" xr:uid="{CFD0AADF-4902-4B28-AE77-0F0DB06EF357}"/>
+    <hyperlink ref="B3" r:id="rId2" display="Patricio2026@" xr:uid="{1B31ABDF-0568-4963-AA52-132C4AEEFDB0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>